<commit_message>
Update on Bug Report Excel
</commit_message>
<xml_diff>
--- a/Bug-Report.xlsx
+++ b/Bug-Report.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ITI\QA\Online-Mobile-Store-WebSite\Test\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\GitFlow-C4-Alex\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8335A87-9E14-42C3-966E-C7B66332A793}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59ACC7AE-6362-44B5-A7A8-D433017007B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -120,9 +120,6 @@
     <t>Empty cart message not appear</t>
   </si>
   <si>
-    <t>no message appear</t>
-  </si>
-  <si>
     <t xml:space="preserve"> message: "Your cart is empty"</t>
   </si>
   <si>
@@ -166,6 +163,9 @@
   </si>
   <si>
     <t>Bug_Supplier_001</t>
+  </si>
+  <si>
+    <t>no message appear ..</t>
   </si>
 </sst>
 </file>
@@ -668,22 +668,22 @@
     </row>
     <row r="4" spans="1:11" ht="102.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>33</v>
-      </c>
       <c r="C4" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>18</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G4" s="5" t="s">
         <v>15</v>
@@ -712,13 +712,13 @@
         <v>28</v>
       </c>
       <c r="D5" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="F5" s="6" t="s">
         <v>30</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>31</v>
       </c>
       <c r="G5" s="5" t="s">
         <v>15</v>
@@ -738,22 +738,22 @@
     </row>
     <row r="6" spans="1:11" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B6" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="F6" s="8" t="s">
         <v>37</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>38</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>15</v>

</xml_diff>